<commit_message>
Update on doc and kicad
</commit_message>
<xml_diff>
--- a/resources/Kururugi-ESC-calculs.xlsx
+++ b/resources/Kururugi-ESC-calculs.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\binon\Desktop\Kururugi-ESC-Dev-Board\resources\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B719D61D-B802-46CC-A52F-B60611813A22}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3B8DDC3F-6373-4753-9F00-32AF70384FF8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" xr2:uid="{A7311F5B-F8BB-4208-8795-7C9379CFEF1C}"/>
   </bookViews>
@@ -1328,7 +1328,7 @@
         <v>0.42033333333333328</v>
       </c>
       <c r="G7" s="6">
-        <f t="shared" si="5"/>
+        <f>$N$9*D7*$N$14</f>
         <v>420.33333333333331</v>
       </c>
       <c r="H7" s="6">

</xml_diff>

<commit_message>
Update doc and kicad
</commit_message>
<xml_diff>
--- a/resources/Kururugi-ESC-calculs.xlsx
+++ b/resources/Kururugi-ESC-calculs.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\binon\Desktop\Kururugi-ESC-Dev-Board\resources\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B1C0B332-76E9-4EB3-8047-242D388BD131}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FBEB0AB0-B861-43F3-8AFC-2947B78D0D78}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" activeTab="3" xr2:uid="{A7311F5B-F8BB-4208-8795-7C9379CFEF1C}"/>
+    <workbookView xWindow="5775" yWindow="-16320" windowWidth="29040" windowHeight="15720" xr2:uid="{A7311F5B-F8BB-4208-8795-7C9379CFEF1C}"/>
   </bookViews>
   <sheets>
     <sheet name="Vsensing computation" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="150" uniqueCount="110">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="177" uniqueCount="137">
   <si>
     <t>R1 (kOhm)</t>
   </si>
@@ -376,10 +376,120 @@
     <t>95% duty is the goal for v1</t>
   </si>
   <si>
-    <t>Dissipation of the mosfet</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Size </t>
+    <t>Vdd (V)</t>
+  </si>
+  <si>
+    <t>Vhbr (V)</t>
+  </si>
+  <si>
+    <t>Vhbh (V)</t>
+  </si>
+  <si>
+    <t>Qg (nC)</t>
+  </si>
+  <si>
+    <t>Ipulldown (mA)</t>
+  </si>
+  <si>
+    <t>Ihbs (mA)</t>
+  </si>
+  <si>
+    <t>Ihb (mA)</t>
+  </si>
+  <si>
+    <t>Fsw min (kHz)</t>
+  </si>
+  <si>
+    <t>Qt (nC)</t>
+  </si>
+  <si>
+    <t>Cbootmin (nC)</t>
+  </si>
+  <si>
+    <t>V0 (V)</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+      </rPr>
+      <t>Δ</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Vbootmax (V)</t>
+    </r>
+  </si>
+  <si>
+    <t>ΔVboot (V)</t>
+  </si>
+  <si>
+    <t>Vddboot (V)</t>
+  </si>
+  <si>
+    <t>C secu (NU)</t>
+  </si>
+  <si>
+    <t>Fmax (kHz)</t>
+  </si>
+  <si>
+    <t>Max duty (%)</t>
+  </si>
+  <si>
+    <t>Toff (µs)</t>
+  </si>
+  <si>
+    <t>Toff secu (NU)</t>
+  </si>
+  <si>
+    <t>Tcharge (µs)</t>
+  </si>
+  <si>
+    <t>Vfinal (V)</t>
+  </si>
+  <si>
+    <r>
+      <t>Rfint (</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+      </rPr>
+      <t>Ω)</t>
+    </r>
+  </si>
+  <si>
+    <t>Rf (Ω)</t>
+  </si>
+  <si>
+    <t>Rfext (Ω)</t>
+  </si>
+  <si>
+    <t>Vf,100mA (V)</t>
+  </si>
+  <si>
+    <t>Vr,100mA (V)</t>
+  </si>
+  <si>
+    <t>Imaxext (A)</t>
+  </si>
+  <si>
+    <t>3Tau (µs)</t>
+  </si>
+  <si>
+    <t>Cboot (nF)</t>
   </si>
 </sst>
 </file>
@@ -392,7 +502,7 @@
     <numFmt numFmtId="166" formatCode="0.000"/>
     <numFmt numFmtId="167" formatCode="0.0"/>
   </numFmts>
-  <fonts count="5" x14ac:knownFonts="1">
+  <fonts count="6" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -428,6 +538,12 @@
       <color theme="1"/>
       <name val="Aptos Narrow"/>
       <family val="2"/>
+    </font>
+    <font>
+      <sz val="8"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="8">
@@ -669,7 +785,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="52">
+  <cellXfs count="48">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -715,9 +831,6 @@
     <xf numFmtId="167" fontId="2" fillId="6" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="2" fontId="2" fillId="6" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="166" fontId="2" fillId="6" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -750,6 +863,13 @@
     <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="167" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="167" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="4" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -771,28 +891,20 @@
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="167" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="167" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="167" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="1" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="2" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="167" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="3">
+  <dxfs count="33">
     <dxf>
       <fill>
         <patternFill>
@@ -814,6 +926,110 @@
         </patternFill>
       </fill>
     </dxf>
+    <dxf>
+      <numFmt numFmtId="167" formatCode="0.0"/>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="2" formatCode="0.00"/>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="167" formatCode="0.0"/>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="167" formatCode="0.0"/>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="167" formatCode="0.0"/>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="167" formatCode="0.0"/>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="167" formatCode="0.0"/>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="2" formatCode="0.00"/>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="1" formatCode="0"/>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="1" formatCode="0"/>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="1" formatCode="0"/>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
@@ -825,6 +1041,75 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{B25A5C38-85C7-4CC9-A2E7-8CC77C0ABABE}" name="Tableau1" displayName="Tableau1" ref="A1:AC3" totalsRowShown="0" dataDxfId="32">
+  <autoFilter ref="A1:AC3" xr:uid="{B25A5C38-85C7-4CC9-A2E7-8CC77C0ABABE}"/>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:AC3">
+    <sortCondition ref="A1:A3"/>
+  </sortState>
+  <tableColumns count="29">
+    <tableColumn id="1" xr3:uid="{8D98E4BE-CBC8-4993-8988-6AA9DD987F18}" name="Vdd (V)" dataDxfId="31"/>
+    <tableColumn id="2" xr3:uid="{9D660013-882C-48E1-9078-C0D5B2A80597}" name="Vf,100mA (V)" dataDxfId="30"/>
+    <tableColumn id="28" xr3:uid="{36BE38BC-4343-43D2-A6AB-DF7CBCB8D288}" name="Vr,100mA (V)" dataDxfId="29">
+      <calculatedColumnFormula>Tableau1[[#This Row],[Rfext (Ω)]]*0.1</calculatedColumnFormula>
+    </tableColumn>
+    <tableColumn id="3" xr3:uid="{3510157E-7A02-4689-8664-3BE0329D115D}" name="Vhbr (V)" dataDxfId="28"/>
+    <tableColumn id="4" xr3:uid="{ECB1DE36-B875-416D-8E2C-DEF25492B782}" name="Vhbh (V)" dataDxfId="27"/>
+    <tableColumn id="5" xr3:uid="{FD7B4A02-8912-4F70-8F8F-E3160EF255C7}" name="ΔVbootmax (V)" dataDxfId="26">
+      <calculatedColumnFormula>A2-B2-D2-E2-Tableau1[[#This Row],[Vr,100mA (V)]]</calculatedColumnFormula>
+    </tableColumn>
+    <tableColumn id="6" xr3:uid="{67DE6560-3A18-4706-8C36-B17ACB24E0A0}" name="Qg (nC)" dataDxfId="25"/>
+    <tableColumn id="7" xr3:uid="{1F6CBA99-F458-419E-95F9-04D2A3D6DC26}" name="Ihb (mA)" dataDxfId="24"/>
+    <tableColumn id="8" xr3:uid="{BABC204A-8EFE-4167-9EF4-887D78DD0CDA}" name="Ihbs (mA)" dataDxfId="23"/>
+    <tableColumn id="9" xr3:uid="{BA788F06-CA53-4E0A-AE4D-896E43A6EDE5}" name="Ipulldown (mA)" dataDxfId="22"/>
+    <tableColumn id="10" xr3:uid="{DB260FB3-06E8-4730-847C-5E6BD063D326}" name="Max duty (%)" dataDxfId="21"/>
+    <tableColumn id="11" xr3:uid="{1CBF1355-D31F-456C-80BE-6CC8C444F650}" name="Fsw min (kHz)" dataDxfId="20"/>
+    <tableColumn id="12" xr3:uid="{1E038DBA-495F-43B9-B606-822FB74520D5}" name="Qt (nC)" dataDxfId="19">
+      <calculatedColumnFormula>(G2*10^-9+H2/L2*10^-6+(I2+J2)/L2*10^-6*K2/100)/10^-9</calculatedColumnFormula>
+    </tableColumn>
+    <tableColumn id="13" xr3:uid="{C79274CC-E2A1-41D2-A761-D54CC7A29829}" name="Cbootmin (nC)" dataDxfId="18">
+      <calculatedColumnFormula>M2/F2</calculatedColumnFormula>
+    </tableColumn>
+    <tableColumn id="14" xr3:uid="{FA3E1CDB-C23D-4FB1-B19E-9DA04D3955EB}" name="C secu (NU)" dataDxfId="17"/>
+    <tableColumn id="15" xr3:uid="{F2329A40-7530-43DD-9A8D-D9481FE6DDA8}" name="Cboot (nF)" dataDxfId="16">
+      <calculatedColumnFormula>N2*O2</calculatedColumnFormula>
+    </tableColumn>
+    <tableColumn id="16" xr3:uid="{E7529637-516C-4BAC-9F9C-F3BCAD77EB6C}" name="ΔVboot (V)" dataDxfId="15">
+      <calculatedColumnFormula>P2/M2</calculatedColumnFormula>
+    </tableColumn>
+    <tableColumn id="17" xr3:uid="{A1106862-E575-4A15-BDC9-291F1DC16EA8}" name="Fmax (kHz)" dataDxfId="14"/>
+    <tableColumn id="18" xr3:uid="{ED56DF9B-39E7-4337-92AA-A19107C957F6}" name="Toff (µs)" dataDxfId="13">
+      <calculatedColumnFormula>1/R2/1000*(1-K2/100)*1000000</calculatedColumnFormula>
+    </tableColumn>
+    <tableColumn id="19" xr3:uid="{5EF5F032-1924-4722-B113-497A8A53F9F9}" name="Toff secu (NU)" dataDxfId="12"/>
+    <tableColumn id="20" xr3:uid="{317078D3-172D-4084-B914-D44E27AF4622}" name="Tcharge (µs)" dataDxfId="11">
+      <calculatedColumnFormula>S2/T2</calculatedColumnFormula>
+    </tableColumn>
+    <tableColumn id="21" xr3:uid="{C74CCBDA-ECD0-48F4-BDD1-B7B52CDCD12C}" name="V0 (V)" dataDxfId="10">
+      <calculatedColumnFormula>A2-B2-Q2-Tableau1[[#This Row],[Vr,100mA (V)]]</calculatedColumnFormula>
+    </tableColumn>
+    <tableColumn id="22" xr3:uid="{24CB70CF-920B-4509-9638-5D3F89476E1B}" name="Vddboot (V)" dataDxfId="9">
+      <calculatedColumnFormula>A2-B2-Tableau1[[#This Row],[Vr,100mA (V)]]</calculatedColumnFormula>
+    </tableColumn>
+    <tableColumn id="23" xr3:uid="{97086D48-76D1-44FE-9798-1E4B672A9D3C}" name="Rfint (Ω)" dataDxfId="8"/>
+    <tableColumn id="25" xr3:uid="{CA25B27B-2081-46A3-A11C-C04EC8E9925A}" name="Rfext (Ω)" dataDxfId="7"/>
+    <tableColumn id="26" xr3:uid="{D571851B-D502-4394-822B-26D2605F0715}" name="Rf (Ω)" dataDxfId="6">
+      <calculatedColumnFormula>IF(Tableau1[[#This Row],[Rfext (Ω)]]&gt;0, 1/(1/Tableau1[[#This Row],[Rfint (Ω)]]+1/Tableau1[[#This Row],[Rfext (Ω)]]), Tableau1[[#This Row],[Rfint (Ω)]])</calculatedColumnFormula>
+    </tableColumn>
+    <tableColumn id="24" xr3:uid="{C72492AB-BD7B-405B-867F-5ADF45417C24}" name="Vfinal (V)" dataDxfId="5">
+      <calculatedColumnFormula>(V2-W2)*EXP(-U2*10^-6/Tableau1[[#This Row],[Rf (Ω)]]/(P2*10^-9))+W2</calculatedColumnFormula>
+    </tableColumn>
+    <tableColumn id="30" xr3:uid="{4A2A1E44-66D8-4309-9DC7-637AF6F8770A}" name="Imaxext (A)" dataDxfId="4">
+      <calculatedColumnFormula>IF(Tableau1[[#This Row],[Rfext (Ω)]]&gt;0,Tableau1[[#This Row],[Vdd (V)]]/Tableau1[[#This Row],[Rfext (Ω)]],0)</calculatedColumnFormula>
+    </tableColumn>
+    <tableColumn id="31" xr3:uid="{B3DB0F25-7B1B-46E1-B7A4-6C280BA75465}" name="3Tau (µs)" dataDxfId="3">
+      <calculatedColumnFormula>IF(Tableau1[[#This Row],[Imaxext (A)]]&gt;0,3*Tableau1[[#This Row],[Rf (Ω)]]*Tableau1[[#This Row],[Cboot (nF)]]*10^-3,0)</calculatedColumnFormula>
+    </tableColumn>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1167,18 +1452,18 @@
   </cols>
   <sheetData>
     <row r="2" spans="2:19" x14ac:dyDescent="0.35">
-      <c r="B2" s="37" t="s">
+      <c r="B2" s="41" t="s">
         <v>61</v>
       </c>
-      <c r="C2" s="38"/>
-      <c r="D2" s="38"/>
-      <c r="E2" s="38"/>
-      <c r="F2" s="38"/>
-      <c r="G2" s="38"/>
-      <c r="H2" s="38"/>
-      <c r="I2" s="38"/>
-      <c r="J2" s="38"/>
-      <c r="K2" s="39"/>
+      <c r="C2" s="42"/>
+      <c r="D2" s="42"/>
+      <c r="E2" s="42"/>
+      <c r="F2" s="42"/>
+      <c r="G2" s="42"/>
+      <c r="H2" s="42"/>
+      <c r="I2" s="42"/>
+      <c r="J2" s="42"/>
+      <c r="K2" s="43"/>
       <c r="M2" s="8" t="s">
         <v>22</v>
       </c>
@@ -2116,11 +2401,11 @@
         <f t="shared" si="4"/>
         <v>3.9062499999999996</v>
       </c>
-      <c r="M19" s="34" t="s">
+      <c r="M19" s="38" t="s">
         <v>25</v>
       </c>
-      <c r="N19" s="35"/>
-      <c r="O19" s="36"/>
+      <c r="N19" s="39"/>
+      <c r="O19" s="40"/>
       <c r="Q19" t="s">
         <v>20</v>
       </c>
@@ -2474,11 +2759,11 @@
       <c r="M26" s="12" t="s">
         <v>32</v>
       </c>
-      <c r="N26" s="33">
+      <c r="N26" s="32">
         <f>R4*N25*1000</f>
         <v>2.0429968393118183</v>
       </c>
-      <c r="O26" s="32" t="s">
+      <c r="O26" s="31" t="s">
         <v>57</v>
       </c>
     </row>
@@ -2742,100 +3027,100 @@
       </c>
     </row>
     <row r="33" spans="2:11" x14ac:dyDescent="0.35">
-      <c r="B33" s="22">
-        <v>1.3068</v>
-      </c>
-      <c r="C33" s="22">
+      <c r="B33" s="21">
+        <v>0.39</v>
+      </c>
+      <c r="C33" s="21">
         <f t="shared" si="11"/>
-        <v>18.295200000000001</v>
-      </c>
-      <c r="D33" s="6">
+        <v>5.4600000000000009</v>
+      </c>
+      <c r="D33" s="20">
         <f t="shared" si="5"/>
-        <v>1.26668</v>
+        <v>0.41100000000000003</v>
       </c>
       <c r="E33" s="20">
         <f t="shared" si="12"/>
-        <v>2.3683961221460827</v>
-      </c>
-      <c r="F33" s="25">
+        <v>7.2992700729926998</v>
+      </c>
+      <c r="F33" s="24">
         <f t="shared" si="2"/>
-        <v>1.26668</v>
+        <v>0.41100000000000003</v>
       </c>
       <c r="G33" s="6">
         <f t="shared" si="8"/>
-        <v>1266.68</v>
+        <v>411</v>
       </c>
       <c r="H33" s="6">
         <f t="shared" si="6"/>
-        <v>1.0925853624325372</v>
+        <v>3.3672896031290667</v>
       </c>
       <c r="I33" s="20">
         <f t="shared" si="13"/>
-        <v>31.884501581471277</v>
+        <v>106.83760683760683</v>
       </c>
       <c r="J33" s="20">
         <f t="shared" si="3"/>
-        <v>2.5507601265177025</v>
+        <v>8.5470085470085468</v>
       </c>
       <c r="K33" s="20">
         <f t="shared" si="4"/>
-        <v>4.7826752372206913</v>
+        <v>16.025641025641022</v>
       </c>
     </row>
     <row r="34" spans="2:11" x14ac:dyDescent="0.35">
-      <c r="B34" s="23"/>
-      <c r="C34" s="23"/>
-      <c r="D34" s="24"/>
-      <c r="E34" s="24"/>
-      <c r="F34" s="26"/>
-      <c r="G34" s="26"/>
-      <c r="H34" s="29"/>
-      <c r="I34" s="24"/>
-      <c r="J34" s="24"/>
-      <c r="K34" s="24"/>
+      <c r="B34" s="22"/>
+      <c r="C34" s="22"/>
+      <c r="D34" s="23"/>
+      <c r="E34" s="23"/>
+      <c r="F34" s="25"/>
+      <c r="G34" s="25"/>
+      <c r="H34" s="28"/>
+      <c r="I34" s="23"/>
+      <c r="J34" s="23"/>
+      <c r="K34" s="23"/>
     </row>
     <row r="35" spans="2:11" x14ac:dyDescent="0.35">
-      <c r="B35" s="22">
-        <v>1.3</v>
-      </c>
-      <c r="C35" s="22">
-        <v>16</v>
+      <c r="B35" s="21">
+        <v>0.39</v>
+      </c>
+      <c r="C35" s="21">
+        <v>5.6</v>
       </c>
       <c r="D35" s="20">
-        <f>B35*C35/(B35+C35)</f>
-        <v>1.2023121387283238</v>
+        <f t="shared" ref="D35" si="14">B35*C35/(B35+C35)+$N$17/1000</f>
+        <v>0.41160767946577625</v>
       </c>
       <c r="E35" s="20">
-        <f>$N$4/D35</f>
-        <v>2.4951923076923075</v>
-      </c>
-      <c r="F35" s="25">
-        <f>IF($N$9=0,$N$23*($N$8+$N$7)*D35,$N$23*(0.1)*D35)</f>
-        <v>1.2023121387283238</v>
+        <f t="shared" ref="E35" si="15">$N$4/D35</f>
+        <v>7.288493751850516</v>
+      </c>
+      <c r="F35" s="24">
+        <f t="shared" ref="F35" si="16">IF($N$9=0,$N$23*($N$8+$N$7)*D35,$N$23*(0.1)*D35)</f>
+        <v>0.41160767946577625</v>
       </c>
       <c r="G35" s="6">
-        <f>C35*D35*$N$14</f>
-        <v>192.36994219653181</v>
-      </c>
-      <c r="H35" s="21">
-        <f>1/(($N$8+$N$7+$N$9)*D35)*1000</f>
-        <v>7.2324414715719065</v>
+        <f t="shared" ref="G35" si="17">$N$9*D35*$N$14</f>
+        <v>411.6076794657763</v>
+      </c>
+      <c r="H35" s="6">
+        <f t="shared" ref="H35" si="18">1/(2*PI()*($N$8+$N$7+$N$9)*D35)*1000</f>
+        <v>3.3623182849316042</v>
       </c>
       <c r="I35" s="20">
-        <f>$N$3*$N$3/(C35+B35)</f>
-        <v>36.127167630057805</v>
+        <f t="shared" ref="I35" si="19">$N$3*$N$3/(C35+B35)</f>
+        <v>104.34056761268782</v>
       </c>
       <c r="J35" s="20">
-        <f>I35*$R$10/1000</f>
-        <v>2.8901734104046244</v>
+        <f t="shared" ref="J35" si="20">I35*$R$10/1000</f>
+        <v>8.3472454090150254</v>
       </c>
       <c r="K35" s="20">
-        <f>I35*$R$11/1000</f>
-        <v>5.4190751445086711</v>
+        <f t="shared" ref="K35" si="21">I35*$R$11/1000</f>
+        <v>15.651085141903174</v>
       </c>
     </row>
     <row r="36" spans="2:11" x14ac:dyDescent="0.35">
-      <c r="G36" s="30"/>
+      <c r="G36" s="29"/>
     </row>
     <row r="37" spans="2:11" x14ac:dyDescent="0.35">
       <c r="F37" s="11" t="s">
@@ -2893,32 +3178,32 @@
   </cols>
   <sheetData>
     <row r="2" spans="2:11" x14ac:dyDescent="0.35">
-      <c r="B2" s="40" t="s">
+      <c r="B2" s="44" t="s">
         <v>62</v>
       </c>
-      <c r="C2" s="40"/>
-      <c r="D2" s="40"/>
-      <c r="E2" s="40"/>
-      <c r="F2" s="40"/>
-      <c r="G2" s="40"/>
+      <c r="C2" s="44"/>
+      <c r="D2" s="44"/>
+      <c r="E2" s="44"/>
+      <c r="F2" s="44"/>
+      <c r="G2" s="44"/>
     </row>
     <row r="3" spans="2:11" x14ac:dyDescent="0.35">
-      <c r="B3" s="27" t="s">
+      <c r="B3" s="26" t="s">
         <v>60</v>
       </c>
-      <c r="C3" s="27" t="s">
+      <c r="C3" s="26" t="s">
         <v>59</v>
       </c>
-      <c r="D3" s="27" t="s">
+      <c r="D3" s="26" t="s">
         <v>58</v>
       </c>
-      <c r="E3" s="27" t="s">
+      <c r="E3" s="26" t="s">
         <v>63</v>
       </c>
-      <c r="F3" s="27" t="s">
+      <c r="F3" s="26" t="s">
         <v>66</v>
       </c>
-      <c r="G3" s="27" t="s">
+      <c r="G3" s="26" t="s">
         <v>67</v>
       </c>
       <c r="I3" s="8" t="s">
@@ -2961,27 +3246,27 @@
       <c r="K4" s="3"/>
     </row>
     <row r="5" spans="2:11" x14ac:dyDescent="0.35">
-      <c r="B5" s="50">
+      <c r="B5" s="9">
         <f>B4+100</f>
         <v>200</v>
       </c>
-      <c r="C5" s="51">
+      <c r="C5" s="6">
         <f t="shared" si="0"/>
         <v>4.2749999999999996E-2</v>
       </c>
-      <c r="D5" s="50">
+      <c r="D5" s="9">
         <f t="shared" si="1"/>
         <v>3</v>
       </c>
-      <c r="E5" s="50">
+      <c r="E5" s="9">
         <f t="shared" si="2"/>
         <v>3.7236363636363636</v>
       </c>
-      <c r="F5" s="50">
+      <c r="F5" s="9">
         <f t="shared" si="3"/>
         <v>238.31272727272727</v>
       </c>
-      <c r="G5" s="51">
+      <c r="G5" s="6">
         <f t="shared" si="4"/>
         <v>62.9425048828125</v>
       </c>
@@ -2996,26 +3281,26 @@
       </c>
     </row>
     <row r="6" spans="2:11" x14ac:dyDescent="0.35">
-      <c r="B6" s="50">
+      <c r="B6" s="9">
         <v>250</v>
       </c>
-      <c r="C6" s="51">
+      <c r="C6" s="6">
         <f t="shared" si="0"/>
         <v>5.3437499999999999E-2</v>
       </c>
-      <c r="D6" s="50">
+      <c r="D6" s="9">
         <f t="shared" si="1"/>
         <v>3.75</v>
       </c>
-      <c r="E6" s="50">
+      <c r="E6" s="9">
         <f t="shared" si="2"/>
         <v>4.6545454545454543</v>
       </c>
-      <c r="F6" s="50">
+      <c r="F6" s="9">
         <f t="shared" si="3"/>
         <v>297.89090909090908</v>
       </c>
-      <c r="G6" s="51">
+      <c r="G6" s="6">
         <f t="shared" si="4"/>
         <v>50.35400390625</v>
       </c>
@@ -3091,27 +3376,27 @@
       </c>
     </row>
     <row r="9" spans="2:11" x14ac:dyDescent="0.35">
-      <c r="B9" s="31">
+      <c r="B9" s="30">
         <f t="shared" si="5"/>
         <v>500</v>
       </c>
-      <c r="C9" s="28">
+      <c r="C9" s="27">
         <f t="shared" si="0"/>
         <v>0.106875</v>
       </c>
-      <c r="D9" s="31">
+      <c r="D9" s="30">
         <f t="shared" si="1"/>
         <v>7.5</v>
       </c>
-      <c r="E9" s="31">
+      <c r="E9" s="30">
         <f t="shared" si="2"/>
         <v>9.3090909090909086</v>
       </c>
-      <c r="F9" s="31">
+      <c r="F9" s="30">
         <f t="shared" si="3"/>
         <v>595.78181818181815</v>
       </c>
-      <c r="G9" s="28">
+      <c r="G9" s="27">
         <f t="shared" si="4"/>
         <v>25.177001953125</v>
       </c>
@@ -3297,7 +3582,7 @@
       <c r="B16" t="s">
         <v>102</v>
       </c>
-      <c r="D16" s="49" t="s">
+      <c r="D16" s="37" t="s">
         <v>104</v>
       </c>
     </row>
@@ -3316,7 +3601,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FE2F4E60-E2C6-48B6-8B32-33733DDD0651}">
-  <dimension ref="B2:P16"/>
+  <dimension ref="B2:N16"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="4.453125" customWidth="1"/>
@@ -3327,8 +3612,8 @@
     <col min="10" max="10" width="30.90625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:16" x14ac:dyDescent="0.35">
-      <c r="B2" s="44" t="s">
+    <row r="2" spans="2:14" x14ac:dyDescent="0.35">
+      <c r="B2" s="34" t="s">
         <v>92</v>
       </c>
       <c r="C2" s="3" t="s">
@@ -3341,8 +3626,8 @@
         <v>52</v>
       </c>
     </row>
-    <row r="3" spans="2:16" x14ac:dyDescent="0.35">
-      <c r="B3" s="44" t="s">
+    <row r="3" spans="2:14" x14ac:dyDescent="0.35">
+      <c r="B3" s="34" t="s">
         <v>81</v>
       </c>
       <c r="C3" s="3" t="s">
@@ -3355,8 +3640,8 @@
         <v>33</v>
       </c>
     </row>
-    <row r="4" spans="2:16" x14ac:dyDescent="0.35">
-      <c r="B4" s="44" t="s">
+    <row r="4" spans="2:14" x14ac:dyDescent="0.35">
+      <c r="B4" s="34" t="s">
         <v>83</v>
       </c>
       <c r="C4" s="3" t="s">
@@ -3369,8 +3654,8 @@
         <v>2</v>
       </c>
     </row>
-    <row r="5" spans="2:16" x14ac:dyDescent="0.35">
-      <c r="B5" s="44" t="s">
+    <row r="5" spans="2:14" x14ac:dyDescent="0.35">
+      <c r="B5" s="34" t="s">
         <v>85</v>
       </c>
       <c r="C5" s="3" t="s">
@@ -3379,12 +3664,12 @@
       <c r="D5" s="3">
         <v>1.2</v>
       </c>
-      <c r="E5" s="41" t="s">
+      <c r="E5" s="3" t="s">
         <v>93</v>
       </c>
     </row>
-    <row r="6" spans="2:16" x14ac:dyDescent="0.35">
-      <c r="B6" s="44" t="s">
+    <row r="6" spans="2:14" x14ac:dyDescent="0.35">
+      <c r="B6" s="34" t="s">
         <v>86</v>
       </c>
       <c r="C6" s="3" t="s">
@@ -3393,15 +3678,12 @@
       <c r="D6" s="3">
         <v>79</v>
       </c>
-      <c r="E6" s="41" t="s">
+      <c r="E6" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="N6" s="42"/>
-      <c r="O6" s="42"/>
-      <c r="P6" s="42"/>
-    </row>
-    <row r="7" spans="2:16" x14ac:dyDescent="0.35">
-      <c r="B7" s="44" t="s">
+    </row>
+    <row r="7" spans="2:14" x14ac:dyDescent="0.35">
+      <c r="B7" s="34" t="s">
         <v>88</v>
       </c>
       <c r="C7" s="3" t="s">
@@ -3410,15 +3692,12 @@
       <c r="D7" s="3">
         <v>81</v>
       </c>
-      <c r="E7" s="41" t="s">
+      <c r="E7" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="N7" s="42"/>
-      <c r="O7" s="42"/>
-      <c r="P7" s="42"/>
-    </row>
-    <row r="8" spans="2:16" x14ac:dyDescent="0.35">
-      <c r="B8" s="44" t="s">
+    </row>
+    <row r="8" spans="2:14" x14ac:dyDescent="0.35">
+      <c r="B8" s="34" t="s">
         <v>90</v>
       </c>
       <c r="C8" s="3" t="s">
@@ -3427,99 +3706,71 @@
       <c r="D8" s="3">
         <v>64</v>
       </c>
-      <c r="E8" s="41" t="s">
+      <c r="E8" s="3" t="s">
         <v>26</v>
       </c>
-      <c r="N8" s="43"/>
-      <c r="O8" s="42"/>
-      <c r="P8" s="42"/>
-    </row>
-    <row r="9" spans="2:16" x14ac:dyDescent="0.35">
-      <c r="N9" s="42"/>
-      <c r="O9" s="42"/>
-      <c r="P9" s="42"/>
-    </row>
-    <row r="10" spans="2:16" x14ac:dyDescent="0.35">
-      <c r="B10" s="44" t="s">
+      <c r="N8" s="33"/>
+    </row>
+    <row r="10" spans="2:14" x14ac:dyDescent="0.35">
+      <c r="B10" s="34" t="s">
         <v>100</v>
       </c>
       <c r="C10" s="3" t="s">
         <v>95</v>
       </c>
-      <c r="D10" s="45">
+      <c r="D10" s="35">
         <f>D5/1000*D2^2*D3/100</f>
         <v>0.25649999999999995</v>
       </c>
       <c r="E10" s="3" t="s">
         <v>96</v>
       </c>
-      <c r="N10" s="42"/>
-      <c r="O10" s="42"/>
-      <c r="P10" s="42"/>
-    </row>
-    <row r="11" spans="2:16" x14ac:dyDescent="0.35">
-      <c r="B11" s="44" t="s">
+    </row>
+    <row r="11" spans="2:14" x14ac:dyDescent="0.35">
+      <c r="B11" s="34" t="s">
         <v>97</v>
       </c>
       <c r="C11" s="3" t="s">
         <v>98</v>
       </c>
-      <c r="D11" s="45">
+      <c r="D11" s="35">
         <f>1/2*D4*D2*(D6+D7)*D8/1000000</f>
         <v>1.9967999999999999</v>
       </c>
       <c r="E11" s="3" t="s">
         <v>96</v>
       </c>
-      <c r="N11" s="42"/>
-      <c r="O11" s="42"/>
-      <c r="P11" s="42"/>
-    </row>
-    <row r="12" spans="2:16" x14ac:dyDescent="0.35">
-      <c r="B12" s="44" t="s">
+    </row>
+    <row r="12" spans="2:14" x14ac:dyDescent="0.35">
+      <c r="B12" s="34" t="s">
         <v>101</v>
       </c>
       <c r="C12" s="3" t="s">
         <v>99</v>
       </c>
-      <c r="D12" s="47">
+      <c r="D12" s="35">
         <f>D10*2+D11</f>
         <v>2.5097999999999998</v>
       </c>
       <c r="E12" s="3" t="s">
         <v>96</v>
       </c>
-      <c r="N12" s="42"/>
-      <c r="O12" s="42"/>
-      <c r="P12" s="42"/>
-    </row>
-    <row r="13" spans="2:16" x14ac:dyDescent="0.35">
-      <c r="B13" s="46"/>
-      <c r="C13" s="46"/>
-      <c r="D13" s="48"/>
-      <c r="E13" s="46"/>
-      <c r="N13" s="42"/>
-      <c r="O13" s="42"/>
-      <c r="P13" s="42"/>
-    </row>
-    <row r="14" spans="2:16" x14ac:dyDescent="0.35">
-      <c r="B14" s="46" t="s">
+    </row>
+    <row r="13" spans="2:14" x14ac:dyDescent="0.35">
+      <c r="D13" s="36"/>
+    </row>
+    <row r="14" spans="2:14" x14ac:dyDescent="0.35">
+      <c r="B14" t="s">
         <v>105</v>
       </c>
-      <c r="N14" s="42"/>
-      <c r="O14" s="42"/>
-      <c r="P14" s="42"/>
-    </row>
-    <row r="15" spans="2:16" x14ac:dyDescent="0.35">
-      <c r="B15" s="46" t="s">
+    </row>
+    <row r="15" spans="2:14" x14ac:dyDescent="0.35">
+      <c r="B15" t="s">
         <v>106</v>
       </c>
-      <c r="N15" s="42"/>
-      <c r="O15" s="42"/>
-      <c r="P15" s="42"/>
-    </row>
-    <row r="16" spans="2:16" x14ac:dyDescent="0.35">
-      <c r="B16" s="46" t="s">
+    </row>
+    <row r="16" spans="2:14" x14ac:dyDescent="0.35">
+      <c r="B16" t="s">
         <v>107</v>
       </c>
     </row>
@@ -3530,20 +3781,334 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D8FD2DCF-3994-4A7C-BD62-D1225B43EB25}">
-  <dimension ref="B2:B4"/>
+  <dimension ref="A1:AC3"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="1" width="9" customWidth="1"/>
+    <col min="2" max="3" width="14" bestFit="1" customWidth="1"/>
+    <col min="4" max="5" width="1.6328125" customWidth="1"/>
+    <col min="6" max="6" width="15.6328125" bestFit="1" customWidth="1"/>
+    <col min="7" max="10" width="1.6328125" customWidth="1"/>
+    <col min="11" max="11" width="13.81640625" customWidth="1"/>
+    <col min="12" max="12" width="1.6328125" customWidth="1"/>
+    <col min="13" max="13" width="9.1796875" customWidth="1"/>
+    <col min="14" max="14" width="16.36328125" customWidth="1"/>
+    <col min="15" max="15" width="13.08984375" customWidth="1"/>
+    <col min="16" max="16" width="12.453125" customWidth="1"/>
+    <col min="17" max="17" width="11.90625" customWidth="1"/>
+    <col min="18" max="18" width="12.26953125" customWidth="1"/>
+    <col min="19" max="20" width="1.6328125" customWidth="1"/>
+    <col min="21" max="21" width="13.36328125" customWidth="1"/>
+    <col min="22" max="22" width="8.1796875" bestFit="1" customWidth="1"/>
+    <col min="23" max="23" width="13" customWidth="1"/>
+    <col min="24" max="24" width="1.6328125" customWidth="1"/>
+    <col min="25" max="25" width="11" bestFit="1" customWidth="1"/>
+    <col min="26" max="26" width="8.26953125" bestFit="1" customWidth="1"/>
+    <col min="27" max="27" width="11" bestFit="1" customWidth="1"/>
+    <col min="28" max="28" width="12.90625" bestFit="1" customWidth="1"/>
+    <col min="29" max="29" width="11" bestFit="1" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="2" spans="2:2" x14ac:dyDescent="0.35">
-      <c r="B2" t="s">
+    <row r="1" spans="1:29" x14ac:dyDescent="0.35">
+      <c r="A1" t="s">
         <v>108</v>
       </c>
-    </row>
-    <row r="4" spans="2:2" x14ac:dyDescent="0.35">
-      <c r="B4" t="s">
+      <c r="B1" t="s">
+        <v>132</v>
+      </c>
+      <c r="C1" t="s">
+        <v>133</v>
+      </c>
+      <c r="D1" t="s">
         <v>109</v>
       </c>
+      <c r="E1" t="s">
+        <v>110</v>
+      </c>
+      <c r="F1" t="s">
+        <v>119</v>
+      </c>
+      <c r="G1" t="s">
+        <v>111</v>
+      </c>
+      <c r="H1" t="s">
+        <v>114</v>
+      </c>
+      <c r="I1" t="s">
+        <v>113</v>
+      </c>
+      <c r="J1" t="s">
+        <v>112</v>
+      </c>
+      <c r="K1" t="s">
+        <v>124</v>
+      </c>
+      <c r="L1" t="s">
+        <v>115</v>
+      </c>
+      <c r="M1" t="s">
+        <v>116</v>
+      </c>
+      <c r="N1" t="s">
+        <v>117</v>
+      </c>
+      <c r="O1" t="s">
+        <v>122</v>
+      </c>
+      <c r="P1" t="s">
+        <v>136</v>
+      </c>
+      <c r="Q1" t="s">
+        <v>120</v>
+      </c>
+      <c r="R1" t="s">
+        <v>123</v>
+      </c>
+      <c r="S1" t="s">
+        <v>125</v>
+      </c>
+      <c r="T1" t="s">
+        <v>126</v>
+      </c>
+      <c r="U1" t="s">
+        <v>127</v>
+      </c>
+      <c r="V1" t="s">
+        <v>118</v>
+      </c>
+      <c r="W1" t="s">
+        <v>121</v>
+      </c>
+      <c r="X1" t="s">
+        <v>129</v>
+      </c>
+      <c r="Y1" t="s">
+        <v>131</v>
+      </c>
+      <c r="Z1" t="s">
+        <v>130</v>
+      </c>
+      <c r="AA1" t="s">
+        <v>128</v>
+      </c>
+      <c r="AB1" t="s">
+        <v>134</v>
+      </c>
+      <c r="AC1" t="s">
+        <v>135</v>
+      </c>
+    </row>
+    <row r="2" spans="1:29" x14ac:dyDescent="0.35">
+      <c r="A2" s="1">
+        <v>10</v>
+      </c>
+      <c r="B2" s="1">
+        <v>0.3</v>
+      </c>
+      <c r="C2" s="1">
+        <f>Tableau1[[#This Row],[Rfext (Ω)]]*0.1</f>
+        <v>0.51</v>
+      </c>
+      <c r="D2" s="1">
+        <v>6</v>
+      </c>
+      <c r="E2" s="1">
+        <v>0.27</v>
+      </c>
+      <c r="F2" s="1">
+        <f>A2-B2-D2-E2-Tableau1[[#This Row],[Vr,100mA (V)]]</f>
+        <v>2.919999999999999</v>
+      </c>
+      <c r="G2" s="1">
+        <v>120</v>
+      </c>
+      <c r="H2" s="1">
+        <v>0.7</v>
+      </c>
+      <c r="I2" s="1">
+        <v>1.25</v>
+      </c>
+      <c r="J2" s="1">
+        <v>1</v>
+      </c>
+      <c r="K2" s="1">
+        <v>95</v>
+      </c>
+      <c r="L2" s="1">
+        <v>24</v>
+      </c>
+      <c r="M2" s="32">
+        <f>(G2*10^-9+H2/L2*10^-6+(I2+J2)/L2*10^-6*K2/100)/10^-9</f>
+        <v>238.22916666666666</v>
+      </c>
+      <c r="N2" s="32">
+        <f>M2/F2</f>
+        <v>81.585331050228334</v>
+      </c>
+      <c r="O2" s="1">
+        <v>2</v>
+      </c>
+      <c r="P2" s="32">
+        <v>300</v>
+      </c>
+      <c r="Q2" s="45">
+        <f>P2/M2</f>
+        <v>1.2592916484477481</v>
+      </c>
+      <c r="R2" s="1">
+        <v>128</v>
+      </c>
+      <c r="S2" s="46">
+        <f>1/R2/1000*(1-K2/100)*1000000</f>
+        <v>0.39062500000000033</v>
+      </c>
+      <c r="T2" s="1">
+        <v>2</v>
+      </c>
+      <c r="U2" s="46">
+        <f>S2/T2</f>
+        <v>0.19531250000000017</v>
+      </c>
+      <c r="V2" s="46">
+        <f>A2-B2-Q2-Tableau1[[#This Row],[Vr,100mA (V)]]</f>
+        <v>7.9307083515522514</v>
+      </c>
+      <c r="W2" s="1">
+        <f>A2-B2-Tableau1[[#This Row],[Vr,100mA (V)]]</f>
+        <v>9.19</v>
+      </c>
+      <c r="X2" s="1">
+        <v>21.5</v>
+      </c>
+      <c r="Y2" s="1">
+        <v>5.0999999999999996</v>
+      </c>
+      <c r="Z2" s="46">
+        <f>IF(Tableau1[[#This Row],[Rfext (Ω)]]&gt;0, 1/(1/Tableau1[[#This Row],[Rfint (Ω)]]+1/Tableau1[[#This Row],[Rfext (Ω)]]), Tableau1[[#This Row],[Rfint (Ω)]])</f>
+        <v>4.1221804511278188</v>
+      </c>
+      <c r="AA2" s="46">
+        <f>(V2-W2)*EXP(-U2*10^-6/Tableau1[[#This Row],[Rf (Ω)]]/(P2*10^-9))+W2</f>
+        <v>8.114685536921213</v>
+      </c>
+      <c r="AB2" s="45">
+        <f>IF(Tableau1[[#This Row],[Rfext (Ω)]]&gt;0,Tableau1[[#This Row],[Vdd (V)]]/Tableau1[[#This Row],[Rfext (Ω)]],0)</f>
+        <v>1.9607843137254903</v>
+      </c>
+      <c r="AC2" s="46">
+        <f>IF(Tableau1[[#This Row],[Imaxext (A)]]&gt;0,3*Tableau1[[#This Row],[Rf (Ω)]]*Tableau1[[#This Row],[Cboot (nF)]]*10^-3,0)</f>
+        <v>3.7099624060150371</v>
+      </c>
+    </row>
+    <row r="3" spans="1:29" x14ac:dyDescent="0.35">
+      <c r="A3" s="1">
+        <v>10</v>
+      </c>
+      <c r="B3" s="1">
+        <v>0.3</v>
+      </c>
+      <c r="C3" s="47">
+        <f>Tableau1[[#This Row],[Rfext (Ω)]]*0.1</f>
+        <v>0.51</v>
+      </c>
+      <c r="D3" s="1">
+        <v>6</v>
+      </c>
+      <c r="E3" s="1">
+        <v>0.27</v>
+      </c>
+      <c r="F3" s="47">
+        <f>A3-B3-D3-E3-Tableau1[[#This Row],[Vr,100mA (V)]]</f>
+        <v>2.919999999999999</v>
+      </c>
+      <c r="G3" s="1">
+        <v>120</v>
+      </c>
+      <c r="H3" s="1">
+        <v>0.7</v>
+      </c>
+      <c r="I3" s="1">
+        <v>1.25</v>
+      </c>
+      <c r="J3" s="1">
+        <v>1</v>
+      </c>
+      <c r="K3" s="1">
+        <v>95</v>
+      </c>
+      <c r="L3" s="1">
+        <v>10</v>
+      </c>
+      <c r="M3" s="32">
+        <f>(G3*10^-9+H3/L3*10^-6+(I3+J3)/L3*10^-6*K3/100)/10^-9</f>
+        <v>403.74999999999994</v>
+      </c>
+      <c r="N3" s="32">
+        <f>M3/F3</f>
+        <v>138.27054794520549</v>
+      </c>
+      <c r="O3" s="1">
+        <v>3</v>
+      </c>
+      <c r="P3" s="32">
+        <f>N3*O3</f>
+        <v>414.81164383561645</v>
+      </c>
+      <c r="Q3" s="45">
+        <f>P3/M3</f>
+        <v>1.0273972602739727</v>
+      </c>
+      <c r="R3" s="1">
+        <v>128</v>
+      </c>
+      <c r="S3" s="46">
+        <f>1/R3/1000*(1-K3/100)*1000000</f>
+        <v>0.39062500000000033</v>
+      </c>
+      <c r="T3" s="1">
+        <v>2</v>
+      </c>
+      <c r="U3" s="46">
+        <f>S3/T3</f>
+        <v>0.19531250000000017</v>
+      </c>
+      <c r="V3" s="46">
+        <f>A3-B3-Q3-Tableau1[[#This Row],[Vr,100mA (V)]]</f>
+        <v>8.1626027397260277</v>
+      </c>
+      <c r="W3" s="47">
+        <f>A3-B3-Tableau1[[#This Row],[Vr,100mA (V)]]</f>
+        <v>9.19</v>
+      </c>
+      <c r="X3" s="1">
+        <v>21.5</v>
+      </c>
+      <c r="Y3" s="1">
+        <v>5.0999999999999996</v>
+      </c>
+      <c r="Z3" s="46">
+        <f>IF(Tableau1[[#This Row],[Rfext (Ω)]]&gt;0, 1/(1/Tableau1[[#This Row],[Rfint (Ω)]]+1/Tableau1[[#This Row],[Rfext (Ω)]]), Tableau1[[#This Row],[Rfint (Ω)]])</f>
+        <v>4.1221804511278188</v>
+      </c>
+      <c r="AA3" s="46">
+        <f>(V3-W3)*EXP(-U3*10^-6/Tableau1[[#This Row],[Rf (Ω)]]/(P3*10^-9))+W3</f>
+        <v>8.2735006704566629</v>
+      </c>
+      <c r="AB3" s="45">
+        <f>IF(Tableau1[[#This Row],[Rfext (Ω)]]&gt;0,Tableau1[[#This Row],[Vdd (V)]]/Tableau1[[#This Row],[Rfext (Ω)]],0)</f>
+        <v>1.9607843137254903</v>
+      </c>
+      <c r="AC3" s="46">
+        <f>IF(Tableau1[[#This Row],[Imaxext (A)]]&gt;0,3*Tableau1[[#This Row],[Rf (Ω)]]*Tableau1[[#This Row],[Cboot (nF)]]*10^-3,0)</f>
+        <v>5.129785347358121</v>
+      </c>
     </row>
   </sheetData>
+  <phoneticPr fontId="5" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
+  <tableParts count="1">
+    <tablePart r:id="rId2"/>
+  </tableParts>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Update kicad and docs
</commit_message>
<xml_diff>
--- a/resources/Kururugi-ESC-calculs.xlsx
+++ b/resources/Kururugi-ESC-calculs.xlsx
@@ -8,15 +8,15 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\binon\Desktop\Kururugi-ESC-Dev-Board\resources\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FBEB0AB0-B861-43F3-8AFC-2947B78D0D78}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{99B2B5A0-7BBE-4CD2-A323-6C36F872F9B2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="5775" yWindow="-16320" windowWidth="29040" windowHeight="15720" xr2:uid="{A7311F5B-F8BB-4208-8795-7C9379CFEF1C}"/>
+    <workbookView xWindow="5775" yWindow="-16320" windowWidth="29040" windowHeight="15720" activeTab="3" xr2:uid="{A7311F5B-F8BB-4208-8795-7C9379CFEF1C}"/>
   </bookViews>
   <sheets>
     <sheet name="Vsensing computation" sheetId="1" r:id="rId1"/>
     <sheet name="Isensing computation" sheetId="2" r:id="rId2"/>
     <sheet name="Mosfet" sheetId="3" r:id="rId3"/>
-    <sheet name="Feuil2" sheetId="4" r:id="rId4"/>
+    <sheet name="GD Cboot" sheetId="4" r:id="rId4"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="177" uniqueCount="137">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="178" uniqueCount="138">
   <si>
     <t>R1 (kOhm)</t>
   </si>
@@ -490,6 +490,9 @@
   </si>
   <si>
     <t>Cboot (nF)</t>
+  </si>
+  <si>
+    <t>dx</t>
   </si>
 </sst>
 </file>
@@ -1429,7 +1432,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{46177FA7-98B1-43B3-8996-93B4082609D4}">
-  <dimension ref="B2:S38"/>
+  <dimension ref="B2:S41"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="3.453125" customWidth="1"/>
@@ -3131,6 +3134,11 @@
     <row r="38" spans="2:11" x14ac:dyDescent="0.35">
       <c r="H38" s="11" t="s">
         <v>41</v>
+      </c>
+    </row>
+    <row r="41" spans="2:11" x14ac:dyDescent="0.35">
+      <c r="H41" t="s">
+        <v>137</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update kicad and doc
</commit_message>
<xml_diff>
--- a/resources/Kururugi-ESC-calculs.xlsx
+++ b/resources/Kururugi-ESC-calculs.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\binon\Desktop\Kururugi-ESC-Dev-Board\resources\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{99B2B5A0-7BBE-4CD2-A323-6C36F872F9B2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{022EFFC5-314D-4BF4-81A0-FE89DAE72F1D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="5775" yWindow="-16320" windowWidth="29040" windowHeight="15720" activeTab="3" xr2:uid="{A7311F5B-F8BB-4208-8795-7C9379CFEF1C}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="178" uniqueCount="138">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="181" uniqueCount="141">
   <si>
     <t>R1 (kOhm)</t>
   </si>
@@ -401,9 +401,6 @@
   </si>
   <si>
     <t>Qt (nC)</t>
-  </si>
-  <si>
-    <t>Cbootmin (nC)</t>
   </si>
   <si>
     <t>V0 (V)</t>
@@ -492,7 +489,19 @@
     <t>Cboot (nF)</t>
   </si>
   <si>
-    <t>dx</t>
+    <t>Cbootmin (nF)</t>
+  </si>
+  <si>
+    <t>Qfreq_max (nC)</t>
+  </si>
+  <si>
+    <t>Max Fsw (kHz)</t>
+  </si>
+  <si>
+    <t>Safety (NU)</t>
+  </si>
+  <si>
+    <t>ImaxIn (mA)</t>
   </si>
 </sst>
 </file>
@@ -788,7 +797,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="48">
+  <cellXfs count="47">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -873,6 +882,12 @@
     <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="167" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="4" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -894,20 +909,15 @@
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="167" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="33">
+  <dxfs count="37">
+    <dxf>
+      <numFmt numFmtId="167" formatCode="0.0"/>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
     <dxf>
       <fill>
         <patternFill>
@@ -928,6 +938,18 @@
           <bgColor rgb="FF92D050"/>
         </patternFill>
       </fill>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="167" formatCode="0.0"/>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="167" formatCode="0.0"/>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="167" formatCode="0.0"/>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
       <numFmt numFmtId="167" formatCode="0.0"/>
@@ -1047,68 +1069,76 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{B25A5C38-85C7-4CC9-A2E7-8CC77C0ABABE}" name="Tableau1" displayName="Tableau1" ref="A1:AC3" totalsRowShown="0" dataDxfId="32">
-  <autoFilter ref="A1:AC3" xr:uid="{B25A5C38-85C7-4CC9-A2E7-8CC77C0ABABE}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{B25A5C38-85C7-4CC9-A2E7-8CC77C0ABABE}" name="Tableau1" displayName="Tableau1" ref="A1:AG3" totalsRowShown="0" dataDxfId="36">
+  <autoFilter ref="A1:AG3" xr:uid="{B25A5C38-85C7-4CC9-A2E7-8CC77C0ABABE}"/>
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:AC3">
     <sortCondition ref="A1:A3"/>
   </sortState>
-  <tableColumns count="29">
-    <tableColumn id="1" xr3:uid="{8D98E4BE-CBC8-4993-8988-6AA9DD987F18}" name="Vdd (V)" dataDxfId="31"/>
-    <tableColumn id="2" xr3:uid="{9D660013-882C-48E1-9078-C0D5B2A80597}" name="Vf,100mA (V)" dataDxfId="30"/>
-    <tableColumn id="28" xr3:uid="{36BE38BC-4343-43D2-A6AB-DF7CBCB8D288}" name="Vr,100mA (V)" dataDxfId="29">
+  <tableColumns count="33">
+    <tableColumn id="1" xr3:uid="{8D98E4BE-CBC8-4993-8988-6AA9DD987F18}" name="Vdd (V)" dataDxfId="35"/>
+    <tableColumn id="2" xr3:uid="{9D660013-882C-48E1-9078-C0D5B2A80597}" name="Vf,100mA (V)" dataDxfId="34"/>
+    <tableColumn id="28" xr3:uid="{36BE38BC-4343-43D2-A6AB-DF7CBCB8D288}" name="Vr,100mA (V)" dataDxfId="33">
       <calculatedColumnFormula>Tableau1[[#This Row],[Rfext (Ω)]]*0.1</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="3" xr3:uid="{3510157E-7A02-4689-8664-3BE0329D115D}" name="Vhbr (V)" dataDxfId="28"/>
-    <tableColumn id="4" xr3:uid="{ECB1DE36-B875-416D-8E2C-DEF25492B782}" name="Vhbh (V)" dataDxfId="27"/>
-    <tableColumn id="5" xr3:uid="{FD7B4A02-8912-4F70-8F8F-E3160EF255C7}" name="ΔVbootmax (V)" dataDxfId="26">
+    <tableColumn id="3" xr3:uid="{3510157E-7A02-4689-8664-3BE0329D115D}" name="Vhbr (V)" dataDxfId="32"/>
+    <tableColumn id="4" xr3:uid="{ECB1DE36-B875-416D-8E2C-DEF25492B782}" name="Vhbh (V)" dataDxfId="31"/>
+    <tableColumn id="5" xr3:uid="{FD7B4A02-8912-4F70-8F8F-E3160EF255C7}" name="ΔVbootmax (V)" dataDxfId="30">
       <calculatedColumnFormula>A2-B2-D2-E2-Tableau1[[#This Row],[Vr,100mA (V)]]</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="6" xr3:uid="{67DE6560-3A18-4706-8C36-B17ACB24E0A0}" name="Qg (nC)" dataDxfId="25"/>
-    <tableColumn id="7" xr3:uid="{1F6CBA99-F458-419E-95F9-04D2A3D6DC26}" name="Ihb (mA)" dataDxfId="24"/>
-    <tableColumn id="8" xr3:uid="{BABC204A-8EFE-4167-9EF4-887D78DD0CDA}" name="Ihbs (mA)" dataDxfId="23"/>
-    <tableColumn id="9" xr3:uid="{BA788F06-CA53-4E0A-AE4D-896E43A6EDE5}" name="Ipulldown (mA)" dataDxfId="22"/>
-    <tableColumn id="10" xr3:uid="{DB260FB3-06E8-4730-847C-5E6BD063D326}" name="Max duty (%)" dataDxfId="21"/>
-    <tableColumn id="11" xr3:uid="{1CBF1355-D31F-456C-80BE-6CC8C444F650}" name="Fsw min (kHz)" dataDxfId="20"/>
-    <tableColumn id="12" xr3:uid="{1E038DBA-495F-43B9-B606-822FB74520D5}" name="Qt (nC)" dataDxfId="19">
+    <tableColumn id="6" xr3:uid="{67DE6560-3A18-4706-8C36-B17ACB24E0A0}" name="Qg (nC)" dataDxfId="29"/>
+    <tableColumn id="7" xr3:uid="{1F6CBA99-F458-419E-95F9-04D2A3D6DC26}" name="Ihb (mA)" dataDxfId="28"/>
+    <tableColumn id="8" xr3:uid="{BABC204A-8EFE-4167-9EF4-887D78DD0CDA}" name="Ihbs (mA)" dataDxfId="27"/>
+    <tableColumn id="9" xr3:uid="{BA788F06-CA53-4E0A-AE4D-896E43A6EDE5}" name="Ipulldown (mA)" dataDxfId="26"/>
+    <tableColumn id="10" xr3:uid="{DB260FB3-06E8-4730-847C-5E6BD063D326}" name="Max duty (%)" dataDxfId="25"/>
+    <tableColumn id="11" xr3:uid="{1CBF1355-D31F-456C-80BE-6CC8C444F650}" name="Fsw min (kHz)" dataDxfId="24"/>
+    <tableColumn id="12" xr3:uid="{1E038DBA-495F-43B9-B606-822FB74520D5}" name="Qt (nC)" dataDxfId="23">
       <calculatedColumnFormula>(G2*10^-9+H2/L2*10^-6+(I2+J2)/L2*10^-6*K2/100)/10^-9</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="13" xr3:uid="{C79274CC-E2A1-41D2-A761-D54CC7A29829}" name="Cbootmin (nC)" dataDxfId="18">
+    <tableColumn id="13" xr3:uid="{C79274CC-E2A1-41D2-A761-D54CC7A29829}" name="Cbootmin (nF)" dataDxfId="22">
       <calculatedColumnFormula>M2/F2</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="14" xr3:uid="{FA3E1CDB-C23D-4FB1-B19E-9DA04D3955EB}" name="C secu (NU)" dataDxfId="17"/>
-    <tableColumn id="15" xr3:uid="{F2329A40-7530-43DD-9A8D-D9481FE6DDA8}" name="Cboot (nF)" dataDxfId="16">
+    <tableColumn id="14" xr3:uid="{FA3E1CDB-C23D-4FB1-B19E-9DA04D3955EB}" name="C secu (NU)" dataDxfId="21"/>
+    <tableColumn id="15" xr3:uid="{F2329A40-7530-43DD-9A8D-D9481FE6DDA8}" name="Cboot (nF)" dataDxfId="20">
       <calculatedColumnFormula>N2*O2</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="16" xr3:uid="{E7529637-516C-4BAC-9F9C-F3BCAD77EB6C}" name="ΔVboot (V)" dataDxfId="15">
+    <tableColumn id="16" xr3:uid="{E7529637-516C-4BAC-9F9C-F3BCAD77EB6C}" name="ΔVboot (V)" dataDxfId="19">
       <calculatedColumnFormula>P2/M2</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="17" xr3:uid="{A1106862-E575-4A15-BDC9-291F1DC16EA8}" name="Fmax (kHz)" dataDxfId="14"/>
-    <tableColumn id="18" xr3:uid="{ED56DF9B-39E7-4337-92AA-A19107C957F6}" name="Toff (µs)" dataDxfId="13">
+    <tableColumn id="17" xr3:uid="{A1106862-E575-4A15-BDC9-291F1DC16EA8}" name="Fmax (kHz)" dataDxfId="18"/>
+    <tableColumn id="18" xr3:uid="{ED56DF9B-39E7-4337-92AA-A19107C957F6}" name="Toff (µs)" dataDxfId="17">
       <calculatedColumnFormula>1/R2/1000*(1-K2/100)*1000000</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="19" xr3:uid="{5EF5F032-1924-4722-B113-497A8A53F9F9}" name="Toff secu (NU)" dataDxfId="12"/>
-    <tableColumn id="20" xr3:uid="{317078D3-172D-4084-B914-D44E27AF4622}" name="Tcharge (µs)" dataDxfId="11">
+    <tableColumn id="19" xr3:uid="{5EF5F032-1924-4722-B113-497A8A53F9F9}" name="Toff secu (NU)" dataDxfId="16"/>
+    <tableColumn id="20" xr3:uid="{317078D3-172D-4084-B914-D44E27AF4622}" name="Tcharge (µs)" dataDxfId="15">
       <calculatedColumnFormula>S2/T2</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="21" xr3:uid="{C74CCBDA-ECD0-48F4-BDD1-B7B52CDCD12C}" name="V0 (V)" dataDxfId="10">
+    <tableColumn id="21" xr3:uid="{C74CCBDA-ECD0-48F4-BDD1-B7B52CDCD12C}" name="V0 (V)" dataDxfId="14">
       <calculatedColumnFormula>A2-B2-Q2-Tableau1[[#This Row],[Vr,100mA (V)]]</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="22" xr3:uid="{24CB70CF-920B-4509-9638-5D3F89476E1B}" name="Vddboot (V)" dataDxfId="9">
+    <tableColumn id="22" xr3:uid="{24CB70CF-920B-4509-9638-5D3F89476E1B}" name="Vddboot (V)" dataDxfId="13">
       <calculatedColumnFormula>A2-B2-Tableau1[[#This Row],[Vr,100mA (V)]]</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="23" xr3:uid="{97086D48-76D1-44FE-9798-1E4B672A9D3C}" name="Rfint (Ω)" dataDxfId="8"/>
-    <tableColumn id="25" xr3:uid="{CA25B27B-2081-46A3-A11C-C04EC8E9925A}" name="Rfext (Ω)" dataDxfId="7"/>
-    <tableColumn id="26" xr3:uid="{D571851B-D502-4394-822B-26D2605F0715}" name="Rf (Ω)" dataDxfId="6">
+    <tableColumn id="23" xr3:uid="{97086D48-76D1-44FE-9798-1E4B672A9D3C}" name="Rfint (Ω)" dataDxfId="12"/>
+    <tableColumn id="25" xr3:uid="{CA25B27B-2081-46A3-A11C-C04EC8E9925A}" name="Rfext (Ω)" dataDxfId="11"/>
+    <tableColumn id="26" xr3:uid="{D571851B-D502-4394-822B-26D2605F0715}" name="Rf (Ω)" dataDxfId="10">
       <calculatedColumnFormula>IF(Tableau1[[#This Row],[Rfext (Ω)]]&gt;0, 1/(1/Tableau1[[#This Row],[Rfint (Ω)]]+1/Tableau1[[#This Row],[Rfext (Ω)]]), Tableau1[[#This Row],[Rfint (Ω)]])</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="24" xr3:uid="{C72492AB-BD7B-405B-867F-5ADF45417C24}" name="Vfinal (V)" dataDxfId="5">
+    <tableColumn id="24" xr3:uid="{C72492AB-BD7B-405B-867F-5ADF45417C24}" name="Vfinal (V)" dataDxfId="9">
       <calculatedColumnFormula>(V2-W2)*EXP(-U2*10^-6/Tableau1[[#This Row],[Rf (Ω)]]/(P2*10^-9))+W2</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="30" xr3:uid="{4A2A1E44-66D8-4309-9DC7-637AF6F8770A}" name="Imaxext (A)" dataDxfId="4">
+    <tableColumn id="30" xr3:uid="{4A2A1E44-66D8-4309-9DC7-637AF6F8770A}" name="Imaxext (A)" dataDxfId="8">
       <calculatedColumnFormula>IF(Tableau1[[#This Row],[Rfext (Ω)]]&gt;0,Tableau1[[#This Row],[Vdd (V)]]/Tableau1[[#This Row],[Rfext (Ω)]],0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="31" xr3:uid="{B3DB0F25-7B1B-46E1-B7A4-6C280BA75465}" name="3Tau (µs)" dataDxfId="3">
+    <tableColumn id="31" xr3:uid="{B3DB0F25-7B1B-46E1-B7A4-6C280BA75465}" name="3Tau (µs)" dataDxfId="7">
       <calculatedColumnFormula>IF(Tableau1[[#This Row],[Imaxext (A)]]&gt;0,3*Tableau1[[#This Row],[Rf (Ω)]]*Tableau1[[#This Row],[Cboot (nF)]]*10^-3,0)</calculatedColumnFormula>
+    </tableColumn>
+    <tableColumn id="27" xr3:uid="{35D08FA4-5098-49A1-96BF-78D1CE0C53DF}" name="Max Fsw (kHz)" dataDxfId="6"/>
+    <tableColumn id="29" xr3:uid="{3AF36601-E787-45F8-A32B-D5DA2AC7BD86}" name="Qfreq_max (nC)" dataDxfId="5">
+      <calculatedColumnFormula>(G2*10^-9+H2/L2*10^-6+(I2+J2)/L2*10^-6*K2/100)/10^-9</calculatedColumnFormula>
+    </tableColumn>
+    <tableColumn id="32" xr3:uid="{35C9A496-3EC8-43C9-89D9-26990B92E82D}" name="Safety (NU)" dataDxfId="4"/>
+    <tableColumn id="33" xr3:uid="{44D3BF9C-C6B6-41CA-BB2A-43E2DA8DB723}" name="ImaxIn (mA)" dataDxfId="0">
+      <calculatedColumnFormula>Tableau1[[#This Row],[Qfreq_max (nC)]]*Tableau1[[#This Row],[Max Fsw (kHz)]]*0.001</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
@@ -1432,7 +1462,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{46177FA7-98B1-43B3-8996-93B4082609D4}">
-  <dimension ref="B2:S41"/>
+  <dimension ref="B2:S38"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="3.453125" customWidth="1"/>
@@ -1455,18 +1485,18 @@
   </cols>
   <sheetData>
     <row r="2" spans="2:19" x14ac:dyDescent="0.35">
-      <c r="B2" s="41" t="s">
+      <c r="B2" s="43" t="s">
         <v>61</v>
       </c>
-      <c r="C2" s="42"/>
-      <c r="D2" s="42"/>
-      <c r="E2" s="42"/>
-      <c r="F2" s="42"/>
-      <c r="G2" s="42"/>
-      <c r="H2" s="42"/>
-      <c r="I2" s="42"/>
-      <c r="J2" s="42"/>
-      <c r="K2" s="43"/>
+      <c r="C2" s="44"/>
+      <c r="D2" s="44"/>
+      <c r="E2" s="44"/>
+      <c r="F2" s="44"/>
+      <c r="G2" s="44"/>
+      <c r="H2" s="44"/>
+      <c r="I2" s="44"/>
+      <c r="J2" s="44"/>
+      <c r="K2" s="45"/>
       <c r="M2" s="8" t="s">
         <v>22</v>
       </c>
@@ -2404,11 +2434,11 @@
         <f t="shared" si="4"/>
         <v>3.9062499999999996</v>
       </c>
-      <c r="M19" s="38" t="s">
+      <c r="M19" s="40" t="s">
         <v>25</v>
       </c>
-      <c r="N19" s="39"/>
-      <c r="O19" s="40"/>
+      <c r="N19" s="41"/>
+      <c r="O19" s="42"/>
       <c r="Q19" t="s">
         <v>20</v>
       </c>
@@ -3136,29 +3166,24 @@
         <v>41</v>
       </c>
     </row>
-    <row r="41" spans="2:11" x14ac:dyDescent="0.35">
-      <c r="H41" t="s">
-        <v>137</v>
-      </c>
-    </row>
   </sheetData>
   <mergeCells count="2">
     <mergeCell ref="M19:O19"/>
     <mergeCell ref="B2:K2"/>
   </mergeCells>
   <conditionalFormatting sqref="F4:F35">
-    <cfRule type="cellIs" dxfId="2" priority="14" operator="between">
+    <cfRule type="cellIs" dxfId="3" priority="14" operator="between">
       <formula>0</formula>
       <formula>$N$22</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="G4:G36">
-    <cfRule type="cellIs" dxfId="1" priority="1" operator="lessThan">
+    <cfRule type="cellIs" dxfId="2" priority="1" operator="lessThan">
       <formula>$N$16</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="H4:H35">
-    <cfRule type="cellIs" dxfId="0" priority="2" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="1" priority="2" operator="greaterThan">
       <formula>$N$10/1000*$N$11</formula>
     </cfRule>
   </conditionalFormatting>
@@ -3186,14 +3211,14 @@
   </cols>
   <sheetData>
     <row r="2" spans="2:11" x14ac:dyDescent="0.35">
-      <c r="B2" s="44" t="s">
+      <c r="B2" s="46" t="s">
         <v>62</v>
       </c>
-      <c r="C2" s="44"/>
-      <c r="D2" s="44"/>
-      <c r="E2" s="44"/>
-      <c r="F2" s="44"/>
-      <c r="G2" s="44"/>
+      <c r="C2" s="46"/>
+      <c r="D2" s="46"/>
+      <c r="E2" s="46"/>
+      <c r="F2" s="46"/>
+      <c r="G2" s="46"/>
     </row>
     <row r="3" spans="2:11" x14ac:dyDescent="0.35">
       <c r="B3" s="26" t="s">
@@ -3789,43 +3814,47 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D8FD2DCF-3994-4A7C-BD62-D1225B43EB25}">
-  <dimension ref="A1:AC3"/>
+  <dimension ref="A1:AG3"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="9" customWidth="1"/>
     <col min="2" max="3" width="14" bestFit="1" customWidth="1"/>
-    <col min="4" max="5" width="1.6328125" customWidth="1"/>
+    <col min="4" max="4" width="1.6328125" customWidth="1"/>
+    <col min="5" max="5" width="1.81640625" customWidth="1"/>
     <col min="6" max="6" width="15.6328125" bestFit="1" customWidth="1"/>
-    <col min="7" max="10" width="1.6328125" customWidth="1"/>
+    <col min="7" max="7" width="4.90625" customWidth="1"/>
+    <col min="8" max="10" width="1.6328125" customWidth="1"/>
     <col min="11" max="11" width="13.81640625" customWidth="1"/>
-    <col min="12" max="12" width="1.6328125" customWidth="1"/>
-    <col min="13" max="13" width="9.1796875" customWidth="1"/>
+    <col min="12" max="12" width="15.6328125" customWidth="1"/>
+    <col min="13" max="13" width="8.6328125" customWidth="1"/>
     <col min="14" max="14" width="16.36328125" customWidth="1"/>
     <col min="15" max="15" width="13.08984375" customWidth="1"/>
     <col min="16" max="16" width="12.453125" customWidth="1"/>
     <col min="17" max="17" width="11.90625" customWidth="1"/>
     <col min="18" max="18" width="12.26953125" customWidth="1"/>
-    <col min="19" max="20" width="1.6328125" customWidth="1"/>
-    <col min="21" max="21" width="13.36328125" customWidth="1"/>
+    <col min="19" max="21" width="6.1796875" customWidth="1"/>
     <col min="22" max="22" width="8.1796875" bestFit="1" customWidth="1"/>
     <col min="23" max="23" width="13" customWidth="1"/>
-    <col min="24" max="24" width="1.6328125" customWidth="1"/>
+    <col min="24" max="24" width="7.81640625" customWidth="1"/>
     <col min="25" max="25" width="11" bestFit="1" customWidth="1"/>
     <col min="26" max="26" width="8.26953125" bestFit="1" customWidth="1"/>
     <col min="27" max="27" width="11" bestFit="1" customWidth="1"/>
     <col min="28" max="28" width="12.90625" bestFit="1" customWidth="1"/>
     <col min="29" max="29" width="11" bestFit="1" customWidth="1"/>
+    <col min="30" max="30" width="16.7265625" bestFit="1" customWidth="1"/>
+    <col min="31" max="31" width="16.7265625" customWidth="1"/>
+    <col min="33" max="33" width="13.453125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:29" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:33" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>108</v>
       </c>
       <c r="B1" t="s">
+        <v>131</v>
+      </c>
+      <c r="C1" t="s">
         <v>132</v>
-      </c>
-      <c r="C1" t="s">
-        <v>133</v>
       </c>
       <c r="D1" t="s">
         <v>109</v>
@@ -3834,7 +3863,7 @@
         <v>110</v>
       </c>
       <c r="F1" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="G1" t="s">
         <v>111</v>
@@ -3849,7 +3878,7 @@
         <v>112</v>
       </c>
       <c r="K1" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="L1" t="s">
         <v>115</v>
@@ -3858,55 +3887,67 @@
         <v>116</v>
       </c>
       <c r="N1" t="s">
+        <v>136</v>
+      </c>
+      <c r="O1" t="s">
+        <v>121</v>
+      </c>
+      <c r="P1" t="s">
+        <v>135</v>
+      </c>
+      <c r="Q1" t="s">
+        <v>119</v>
+      </c>
+      <c r="R1" t="s">
+        <v>122</v>
+      </c>
+      <c r="S1" t="s">
+        <v>124</v>
+      </c>
+      <c r="T1" t="s">
+        <v>125</v>
+      </c>
+      <c r="U1" t="s">
+        <v>126</v>
+      </c>
+      <c r="V1" t="s">
         <v>117</v>
       </c>
-      <c r="O1" t="s">
-        <v>122</v>
-      </c>
-      <c r="P1" t="s">
-        <v>136</v>
-      </c>
-      <c r="Q1" t="s">
+      <c r="W1" t="s">
         <v>120</v>
       </c>
-      <c r="R1" t="s">
-        <v>123</v>
-      </c>
-      <c r="S1" t="s">
-        <v>125</v>
-      </c>
-      <c r="T1" t="s">
-        <v>126</v>
-      </c>
-      <c r="U1" t="s">
+      <c r="X1" t="s">
+        <v>128</v>
+      </c>
+      <c r="Y1" t="s">
+        <v>130</v>
+      </c>
+      <c r="Z1" t="s">
+        <v>129</v>
+      </c>
+      <c r="AA1" t="s">
         <v>127</v>
       </c>
-      <c r="V1" t="s">
-        <v>118</v>
-      </c>
-      <c r="W1" t="s">
-        <v>121</v>
-      </c>
-      <c r="X1" t="s">
-        <v>129</v>
-      </c>
-      <c r="Y1" t="s">
-        <v>131</v>
-      </c>
-      <c r="Z1" t="s">
-        <v>130</v>
-      </c>
-      <c r="AA1" t="s">
-        <v>128</v>
-      </c>
       <c r="AB1" t="s">
+        <v>133</v>
+      </c>
+      <c r="AC1" t="s">
         <v>134</v>
       </c>
-      <c r="AC1" t="s">
-        <v>135</v>
-      </c>
-    </row>
-    <row r="2" spans="1:29" x14ac:dyDescent="0.35">
+      <c r="AD1" t="s">
+        <v>138</v>
+      </c>
+      <c r="AE1" t="s">
+        <v>137</v>
+      </c>
+      <c r="AF1" t="s">
+        <v>139</v>
+      </c>
+      <c r="AG1" t="s">
+        <v>140</v>
+      </c>
+    </row>
+    <row r="2" spans="1:33" x14ac:dyDescent="0.35">
       <c r="A2" s="1">
         <v>10</v>
       </c>
@@ -3959,25 +4000,25 @@
       <c r="P2" s="32">
         <v>300</v>
       </c>
-      <c r="Q2" s="45">
+      <c r="Q2" s="38">
         <f>P2/M2</f>
         <v>1.2592916484477481</v>
       </c>
       <c r="R2" s="1">
         <v>128</v>
       </c>
-      <c r="S2" s="46">
+      <c r="S2" s="39">
         <f>1/R2/1000*(1-K2/100)*1000000</f>
         <v>0.39062500000000033</v>
       </c>
       <c r="T2" s="1">
         <v>2</v>
       </c>
-      <c r="U2" s="46">
+      <c r="U2" s="39">
         <f>S2/T2</f>
         <v>0.19531250000000017</v>
       </c>
-      <c r="V2" s="46">
+      <c r="V2" s="39">
         <f>A2-B2-Q2-Tableau1[[#This Row],[Vr,100mA (V)]]</f>
         <v>7.9307083515522514</v>
       </c>
@@ -3991,31 +4032,45 @@
       <c r="Y2" s="1">
         <v>5.0999999999999996</v>
       </c>
-      <c r="Z2" s="46">
+      <c r="Z2" s="39">
         <f>IF(Tableau1[[#This Row],[Rfext (Ω)]]&gt;0, 1/(1/Tableau1[[#This Row],[Rfint (Ω)]]+1/Tableau1[[#This Row],[Rfext (Ω)]]), Tableau1[[#This Row],[Rfint (Ω)]])</f>
         <v>4.1221804511278188</v>
       </c>
-      <c r="AA2" s="46">
+      <c r="AA2" s="39">
         <f>(V2-W2)*EXP(-U2*10^-6/Tableau1[[#This Row],[Rf (Ω)]]/(P2*10^-9))+W2</f>
         <v>8.114685536921213</v>
       </c>
-      <c r="AB2" s="45">
+      <c r="AB2" s="38">
         <f>IF(Tableau1[[#This Row],[Rfext (Ω)]]&gt;0,Tableau1[[#This Row],[Vdd (V)]]/Tableau1[[#This Row],[Rfext (Ω)]],0)</f>
         <v>1.9607843137254903</v>
       </c>
-      <c r="AC2" s="46">
+      <c r="AC2" s="39">
         <f>IF(Tableau1[[#This Row],[Imaxext (A)]]&gt;0,3*Tableau1[[#This Row],[Rf (Ω)]]*Tableau1[[#This Row],[Cboot (nF)]]*10^-3,0)</f>
         <v>3.7099624060150371</v>
       </c>
-    </row>
-    <row r="3" spans="1:29" x14ac:dyDescent="0.35">
+      <c r="AD2" s="39">
+        <v>128</v>
+      </c>
+      <c r="AE2" s="39">
+        <f>(G2*10^-9+H2/L2*10^-6+(I2+J2)/L2*10^-6*K2/100)/10^-9</f>
+        <v>238.22916666666666</v>
+      </c>
+      <c r="AF2" s="39">
+        <v>2</v>
+      </c>
+      <c r="AG2" s="39">
+        <f>Tableau1[[#This Row],[Qfreq_max (nC)]]*Tableau1[[#This Row],[Max Fsw (kHz)]]*0.001</f>
+        <v>30.493333333333332</v>
+      </c>
+    </row>
+    <row r="3" spans="1:33" x14ac:dyDescent="0.35">
       <c r="A3" s="1">
         <v>10</v>
       </c>
       <c r="B3" s="1">
         <v>0.3</v>
       </c>
-      <c r="C3" s="47">
+      <c r="C3" s="1">
         <f>Tableau1[[#This Row],[Rfext (Ω)]]*0.1</f>
         <v>0.51</v>
       </c>
@@ -4025,7 +4080,7 @@
       <c r="E3" s="1">
         <v>0.27</v>
       </c>
-      <c r="F3" s="47">
+      <c r="F3" s="1">
         <f>A3-B3-D3-E3-Tableau1[[#This Row],[Vr,100mA (V)]]</f>
         <v>2.919999999999999</v>
       </c>
@@ -4045,46 +4100,46 @@
         <v>95</v>
       </c>
       <c r="L3" s="1">
-        <v>10</v>
+        <v>24</v>
       </c>
       <c r="M3" s="32">
         <f>(G3*10^-9+H3/L3*10^-6+(I3+J3)/L3*10^-6*K3/100)/10^-9</f>
-        <v>403.74999999999994</v>
+        <v>238.22916666666666</v>
       </c>
       <c r="N3" s="32">
         <f>M3/F3</f>
-        <v>138.27054794520549</v>
+        <v>81.585331050228334</v>
       </c>
       <c r="O3" s="1">
         <v>3</v>
       </c>
       <c r="P3" s="32">
         <f>N3*O3</f>
-        <v>414.81164383561645</v>
-      </c>
-      <c r="Q3" s="45">
+        <v>244.75599315068501</v>
+      </c>
+      <c r="Q3" s="38">
         <f>P3/M3</f>
-        <v>1.0273972602739727</v>
+        <v>1.0273972602739729</v>
       </c>
       <c r="R3" s="1">
         <v>128</v>
       </c>
-      <c r="S3" s="46">
+      <c r="S3" s="39">
         <f>1/R3/1000*(1-K3/100)*1000000</f>
         <v>0.39062500000000033</v>
       </c>
       <c r="T3" s="1">
         <v>2</v>
       </c>
-      <c r="U3" s="46">
+      <c r="U3" s="39">
         <f>S3/T3</f>
         <v>0.19531250000000017</v>
       </c>
-      <c r="V3" s="46">
+      <c r="V3" s="39">
         <f>A3-B3-Q3-Tableau1[[#This Row],[Vr,100mA (V)]]</f>
-        <v>8.1626027397260277</v>
-      </c>
-      <c r="W3" s="47">
+        <v>8.1626027397260259</v>
+      </c>
+      <c r="W3" s="1">
         <f>A3-B3-Tableau1[[#This Row],[Vr,100mA (V)]]</f>
         <v>9.19</v>
       </c>
@@ -4094,21 +4149,35 @@
       <c r="Y3" s="1">
         <v>5.0999999999999996</v>
       </c>
-      <c r="Z3" s="46">
+      <c r="Z3" s="39">
         <f>IF(Tableau1[[#This Row],[Rfext (Ω)]]&gt;0, 1/(1/Tableau1[[#This Row],[Rfint (Ω)]]+1/Tableau1[[#This Row],[Rfext (Ω)]]), Tableau1[[#This Row],[Rfint (Ω)]])</f>
         <v>4.1221804511278188</v>
       </c>
-      <c r="AA3" s="46">
+      <c r="AA3" s="39">
         <f>(V3-W3)*EXP(-U3*10^-6/Tableau1[[#This Row],[Rf (Ω)]]/(P3*10^-9))+W3</f>
-        <v>8.2735006704566629</v>
-      </c>
-      <c r="AB3" s="45">
+        <v>8.3434241159982783</v>
+      </c>
+      <c r="AB3" s="38">
         <f>IF(Tableau1[[#This Row],[Rfext (Ω)]]&gt;0,Tableau1[[#This Row],[Vdd (V)]]/Tableau1[[#This Row],[Rfext (Ω)]],0)</f>
         <v>1.9607843137254903</v>
       </c>
-      <c r="AC3" s="46">
+      <c r="AC3" s="39">
         <f>IF(Tableau1[[#This Row],[Imaxext (A)]]&gt;0,3*Tableau1[[#This Row],[Rf (Ω)]]*Tableau1[[#This Row],[Cboot (nF)]]*10^-3,0)</f>
-        <v>5.129785347358121</v>
+        <v>3.0267851107863843</v>
+      </c>
+      <c r="AD3" s="39">
+        <v>128</v>
+      </c>
+      <c r="AE3" s="39">
+        <f>(G3*10^-9+H3/L3*10^-6+(I3+J3)/L3*10^-6*K3/100)/10^-9</f>
+        <v>238.22916666666666</v>
+      </c>
+      <c r="AF3" s="39">
+        <v>2</v>
+      </c>
+      <c r="AG3" s="39">
+        <f>Tableau1[[#This Row],[Qfreq_max (nC)]]*Tableau1[[#This Row],[Max Fsw (kHz)]]*0.001</f>
+        <v>30.493333333333332</v>
       </c>
     </row>
   </sheetData>

</xml_diff>